<commit_message>
Mise à jour les vues et fichiers csv
</commit_message>
<xml_diff>
--- a/exports/xlsx/KPI_HOSPITALISATION.xlsx
+++ b/exports/xlsx/KPI_HOSPITALISATION.xlsx
@@ -17,8 +17,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -429,13 +429,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MOIS</t>
+          <t>JOUR</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -486,31 +486,31 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46113</v>
+        <v>46141</v>
       </c>
       <c r="B2" t="n">
-        <v>1316</v>
+        <v>498</v>
       </c>
       <c r="C2" t="n">
-        <v>1316</v>
+        <v>498</v>
       </c>
       <c r="D2" t="n">
         <v>67</v>
       </c>
       <c r="E2" t="n">
-        <v>5.354863</v>
+        <v>5.26506</v>
       </c>
       <c r="F2" t="n">
-        <v>104482.42</v>
+        <v>38668.75</v>
       </c>
       <c r="G2" t="n">
-        <v>79.39393617021277</v>
+        <v>77.64809236947791</v>
       </c>
       <c r="H2" t="n">
-        <v>632</v>
+        <v>374</v>
       </c>
       <c r="I2" t="n">
-        <v>1316</v>
+        <v>498</v>
       </c>
       <c r="J2" t="n">
         <v>100</v>
@@ -518,33 +518,353 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B3" t="n">
+        <v>818</v>
+      </c>
+      <c r="C3" t="n">
+        <v>818</v>
+      </c>
+      <c r="D3" t="n">
+        <v>67</v>
+      </c>
+      <c r="E3" t="n">
+        <v>5.409535</v>
+      </c>
+      <c r="F3" t="n">
+        <v>65813.67</v>
+      </c>
+      <c r="G3" t="n">
+        <v>80.45680929095354</v>
+      </c>
+      <c r="H3" t="n">
+        <v>508</v>
+      </c>
+      <c r="I3" t="n">
+        <v>818</v>
+      </c>
+      <c r="J3" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
         <v>46143</v>
       </c>
-      <c r="B3" t="n">
-        <v>9446</v>
-      </c>
-      <c r="C3" t="n">
-        <v>9446</v>
-      </c>
-      <c r="D3" t="n">
-        <v>67</v>
-      </c>
-      <c r="E3" t="n">
-        <v>5.337286</v>
-      </c>
-      <c r="F3" t="n">
-        <v>742785.67</v>
-      </c>
-      <c r="G3" t="n">
-        <v>78.63494283294517</v>
-      </c>
-      <c r="H3" t="n">
-        <v>787</v>
-      </c>
-      <c r="I3" t="n">
-        <v>9446</v>
-      </c>
-      <c r="J3" t="n">
+      <c r="B4" t="n">
+        <v>472</v>
+      </c>
+      <c r="C4" t="n">
+        <v>472</v>
+      </c>
+      <c r="D4" t="n">
+        <v>67</v>
+      </c>
+      <c r="E4" t="n">
+        <v>4.980932</v>
+      </c>
+      <c r="F4" t="n">
+        <v>35916.31</v>
+      </c>
+      <c r="G4" t="n">
+        <v>76.09387711864406</v>
+      </c>
+      <c r="H4" t="n">
+        <v>359</v>
+      </c>
+      <c r="I4" t="n">
+        <v>472</v>
+      </c>
+      <c r="J4" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B5" t="n">
+        <v>450</v>
+      </c>
+      <c r="C5" t="n">
+        <v>450</v>
+      </c>
+      <c r="D5" t="n">
+        <v>67</v>
+      </c>
+      <c r="E5" t="n">
+        <v>5.284444</v>
+      </c>
+      <c r="F5" t="n">
+        <v>34731.41</v>
+      </c>
+      <c r="G5" t="n">
+        <v>77.18091111111112</v>
+      </c>
+      <c r="H5" t="n">
+        <v>333</v>
+      </c>
+      <c r="I5" t="n">
+        <v>450</v>
+      </c>
+      <c r="J5" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B6" t="n">
+        <v>1289</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1289</v>
+      </c>
+      <c r="D6" t="n">
+        <v>67</v>
+      </c>
+      <c r="E6" t="n">
+        <v>5.632273</v>
+      </c>
+      <c r="F6" t="n">
+        <v>106670.94</v>
+      </c>
+      <c r="G6" t="n">
+        <v>82.75480217222653</v>
+      </c>
+      <c r="H6" t="n">
+        <v>638</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1289</v>
+      </c>
+      <c r="J6" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B7" t="n">
+        <v>445</v>
+      </c>
+      <c r="C7" t="n">
+        <v>445</v>
+      </c>
+      <c r="D7" t="n">
+        <v>67</v>
+      </c>
+      <c r="E7" t="n">
+        <v>5.739326</v>
+      </c>
+      <c r="F7" t="n">
+        <v>36802.53</v>
+      </c>
+      <c r="G7" t="n">
+        <v>82.70231460674157</v>
+      </c>
+      <c r="H7" t="n">
+        <v>330</v>
+      </c>
+      <c r="I7" t="n">
+        <v>445</v>
+      </c>
+      <c r="J7" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B8" t="n">
+        <v>1128</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1128</v>
+      </c>
+      <c r="D8" t="n">
+        <v>67</v>
+      </c>
+      <c r="E8" t="n">
+        <v>5.049645</v>
+      </c>
+      <c r="F8" t="n">
+        <v>85395.23</v>
+      </c>
+      <c r="G8" t="n">
+        <v>75.70499113475177</v>
+      </c>
+      <c r="H8" t="n">
+        <v>594</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1128</v>
+      </c>
+      <c r="J8" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B9" t="n">
+        <v>1170</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1170</v>
+      </c>
+      <c r="D9" t="n">
+        <v>67</v>
+      </c>
+      <c r="E9" t="n">
+        <v>5.27265</v>
+      </c>
+      <c r="F9" t="n">
+        <v>90432.50999999999</v>
+      </c>
+      <c r="G9" t="n">
+        <v>77.29274358974358</v>
+      </c>
+      <c r="H9" t="n">
+        <v>612</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1170</v>
+      </c>
+      <c r="J9" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B10" t="n">
+        <v>1256</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1256</v>
+      </c>
+      <c r="D10" t="n">
+        <v>67</v>
+      </c>
+      <c r="E10" t="n">
+        <v>5.545382</v>
+      </c>
+      <c r="F10" t="n">
+        <v>101032.2</v>
+      </c>
+      <c r="G10" t="n">
+        <v>80.43964968152866</v>
+      </c>
+      <c r="H10" t="n">
+        <v>625</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1256</v>
+      </c>
+      <c r="J10" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>46150</v>
+      </c>
+      <c r="B11" t="n">
+        <v>1371</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1371</v>
+      </c>
+      <c r="D11" t="n">
+        <v>67</v>
+      </c>
+      <c r="E11" t="n">
+        <v>5.390956</v>
+      </c>
+      <c r="F11" t="n">
+        <v>108258.19</v>
+      </c>
+      <c r="G11" t="n">
+        <v>78.96293946024799</v>
+      </c>
+      <c r="H11" t="n">
+        <v>649</v>
+      </c>
+      <c r="I11" t="n">
+        <v>1371</v>
+      </c>
+      <c r="J11" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B12" t="n">
+        <v>476</v>
+      </c>
+      <c r="C12" t="n">
+        <v>476</v>
+      </c>
+      <c r="D12" t="n">
+        <v>67</v>
+      </c>
+      <c r="E12" t="n">
+        <v>4.747899</v>
+      </c>
+      <c r="F12" t="n">
+        <v>33712.13</v>
+      </c>
+      <c r="G12" t="n">
+        <v>70.8238025210084</v>
+      </c>
+      <c r="H12" t="n">
+        <v>357</v>
+      </c>
+      <c r="I12" t="n">
+        <v>476</v>
+      </c>
+      <c r="J12" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B13" t="n">
+        <v>1389</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1389</v>
+      </c>
+      <c r="D13" t="n">
+        <v>67</v>
+      </c>
+      <c r="E13" t="n">
+        <v>5.321814</v>
+      </c>
+      <c r="F13" t="n">
+        <v>109834.22</v>
+      </c>
+      <c r="G13" t="n">
+        <v>79.07431245500361</v>
+      </c>
+      <c r="H13" t="n">
+        <v>637</v>
+      </c>
+      <c r="I13" t="n">
+        <v>1389</v>
+      </c>
+      <c r="J13" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>